<commit_message>
chore: save changes and finalize project updates
</commit_message>
<xml_diff>
--- a/docs/BCCC_CNPM/TERENCE_TestExecution.xlsx
+++ b/docs/BCCC_CNPM/TERENCE_TestExecution.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Hutech\Congnghephanmem\TERENCE\TERENCE-main\docs\BCCC_CNPM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09254AA2-5AEF-4CE2-AF76-072C4CB6D433}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{055F6359-27E4-4CDE-ADBA-2633FDB3CB70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_Summary" sheetId="1" r:id="rId1"/>
@@ -2889,9 +2889,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3232,9 +3235,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L22"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3247,7 +3250,7 @@
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
     </row>
-    <row r="3" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -3255,7 +3258,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3263,7 +3266,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -3271,7 +3274,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -3279,7 +3282,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3287,7 +3290,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -3295,7 +3298,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -3303,7 +3306,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -3338,7 +3341,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -3346,7 +3349,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -3354,7 +3357,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>30</v>
       </c>
@@ -3362,7 +3365,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -3370,7 +3373,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>34</v>
       </c>
@@ -3378,7 +3381,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>36</v>
       </c>
@@ -3386,7 +3389,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>38</v>
       </c>
@@ -3394,7 +3397,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>40</v>
       </c>
@@ -3402,7 +3405,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="H19" t="s">
         <v>42</v>
       </c>
@@ -3413,7 +3416,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="H20" t="s">
         <v>45</v>
       </c>
@@ -3421,7 +3424,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="H21" t="s">
         <v>47</v>
       </c>
@@ -3429,7 +3432,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="H22" t="s">
         <v>49</v>
       </c>
@@ -3452,17 +3455,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AE19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.69921875" customWidth="1"/>
     <col min="2" max="2" width="18.69921875" customWidth="1"/>
     <col min="3" max="3" width="17.296875" customWidth="1"/>
     <col min="4" max="4" width="23.09765625" customWidth="1"/>
-    <col min="5" max="5" width="19.69921875" customWidth="1"/>
-    <col min="6" max="6" width="12.3984375" customWidth="1"/>
+    <col min="5" max="5" width="28.3984375" customWidth="1"/>
+    <col min="6" max="6" width="35.3984375" customWidth="1"/>
+    <col min="7" max="7" width="29.59765625" customWidth="1"/>
+    <col min="22" max="22" width="17.09765625" customWidth="1"/>
+    <col min="23" max="23" width="17.8984375" customWidth="1"/>
+    <col min="24" max="24" width="13.796875" customWidth="1"/>
+    <col min="25" max="25" width="13.19921875" customWidth="1"/>
+    <col min="27" max="27" width="19.69921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>51</v>
       </c>
@@ -3485,7 +3494,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -3508,7 +3517,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
         <v>60</v>
       </c>
@@ -3517,19 +3526,19 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
         <v>61</v>
       </c>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>62</v>
       </c>
       <c r="D5" s="1"/>
     </row>
-    <row r="6" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="I6" s="1" t="s">
         <v>63</v>
       </c>
@@ -3541,7 +3550,7 @@
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
     </row>
-    <row r="7" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>64</v>
       </c>
@@ -3636,7 +3645,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="8" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:31" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>92</v>
       </c>
@@ -3652,7 +3661,7 @@
       <c r="E8" t="s">
         <v>96</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="2" t="s">
         <v>97</v>
       </c>
       <c r="G8" t="s">
@@ -3707,7 +3716,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:31" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>106</v>
       </c>
@@ -3723,7 +3732,7 @@
       <c r="E9" t="s">
         <v>109</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="2" t="s">
         <v>110</v>
       </c>
       <c r="G9" t="s">
@@ -3778,7 +3787,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:31" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>113</v>
       </c>
@@ -3794,7 +3803,7 @@
       <c r="E10" t="s">
         <v>109</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="2" t="s">
         <v>115</v>
       </c>
       <c r="G10" t="s">
@@ -3849,7 +3858,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:31" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>118</v>
       </c>
@@ -3865,7 +3874,7 @@
       <c r="E11" t="s">
         <v>109</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="2" t="s">
         <v>120</v>
       </c>
       <c r="G11" t="s">
@@ -3920,7 +3929,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:31" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>123</v>
       </c>
@@ -3936,7 +3945,7 @@
       <c r="E12" t="s">
         <v>96</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="2" t="s">
         <v>126</v>
       </c>
       <c r="G12" t="s">
@@ -3991,7 +4000,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="13" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:31" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>129</v>
       </c>
@@ -4007,7 +4016,7 @@
       <c r="E13" t="s">
         <v>131</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="2" t="s">
         <v>132</v>
       </c>
       <c r="G13" t="s">
@@ -4062,7 +4071,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:31" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>135</v>
       </c>
@@ -4078,7 +4087,7 @@
       <c r="E14" t="s">
         <v>138</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="2" t="s">
         <v>139</v>
       </c>
       <c r="G14" t="s">
@@ -4133,7 +4142,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:31" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>142</v>
       </c>
@@ -4149,7 +4158,7 @@
       <c r="E15" t="s">
         <v>109</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="2" t="s">
         <v>145</v>
       </c>
       <c r="G15" t="s">
@@ -4204,7 +4213,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>148</v>
       </c>
@@ -4275,7 +4284,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:31" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>155</v>
       </c>
@@ -4291,7 +4300,7 @@
       <c r="E17" t="s">
         <v>158</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="2" t="s">
         <v>159</v>
       </c>
       <c r="G17" t="s">
@@ -4346,7 +4355,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>161</v>
       </c>
@@ -4417,7 +4426,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>167</v>
       </c>
@@ -4500,7 +4509,7 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:AE7 A20:AE200 A8:V8 X8:AE8 A9:V19 X9:AE19" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:AE7 A20:AE200 A8:E8 X8:AE8 A16:V16 X9:AE19 A9:E9 G9:V9 G8:V8 A10:E10 G10:V10 A11:E11 G11:V11 A12:E12 G12:V12 A13:E13 G13:V13 A14:E14 G14:V14 A15:E15 G15:V15 A18:V19 A17:E17 G17:V17" numberStoredAsText="1"/>
   </ignoredErrors>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
@@ -4509,9 +4518,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:AE17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>720</v>
       </c>
@@ -4534,7 +4543,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -4557,7 +4566,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
         <v>60</v>
       </c>
@@ -4566,19 +4575,19 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
         <v>61</v>
       </c>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>62</v>
       </c>
       <c r="D5" s="1"/>
     </row>
-    <row r="6" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="I6" s="1" t="s">
         <v>63</v>
       </c>
@@ -4590,7 +4599,7 @@
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
     </row>
-    <row r="7" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>64</v>
       </c>
@@ -4685,7 +4694,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="8" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>174</v>
       </c>
@@ -4756,7 +4765,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>180</v>
       </c>
@@ -4827,7 +4836,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>186</v>
       </c>
@@ -4898,7 +4907,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>189</v>
       </c>
@@ -4969,7 +4978,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>194</v>
       </c>
@@ -5040,7 +5049,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="13" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>199</v>
       </c>
@@ -5111,7 +5120,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>204</v>
       </c>
@@ -5182,7 +5191,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>210</v>
       </c>
@@ -5253,7 +5262,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>215</v>
       </c>
@@ -5324,7 +5333,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>220</v>
       </c>
@@ -5416,9 +5425,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:AE21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>51</v>
       </c>
@@ -5441,7 +5450,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -5464,7 +5473,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
         <v>60</v>
       </c>
@@ -5473,19 +5482,19 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
         <v>61</v>
       </c>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>62</v>
       </c>
       <c r="D5" s="1"/>
     </row>
-    <row r="6" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="I6" s="1" t="s">
         <v>63</v>
       </c>
@@ -5497,7 +5506,7 @@
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
     </row>
-    <row r="7" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>64</v>
       </c>
@@ -5592,7 +5601,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="8" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>227</v>
       </c>
@@ -5663,7 +5672,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>234</v>
       </c>
@@ -5734,7 +5743,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>241</v>
       </c>
@@ -5805,7 +5814,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>247</v>
       </c>
@@ -5876,7 +5885,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="12" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>259</v>
       </c>
@@ -5947,7 +5956,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="13" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>265</v>
       </c>
@@ -6018,7 +6027,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>273</v>
       </c>
@@ -6089,7 +6098,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>280</v>
       </c>
@@ -6160,7 +6169,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>288</v>
       </c>
@@ -6231,7 +6240,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>295</v>
       </c>
@@ -6302,7 +6311,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>302</v>
       </c>
@@ -6373,7 +6382,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>309</v>
       </c>
@@ -6444,7 +6453,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="20" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>316</v>
       </c>
@@ -6515,7 +6524,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="21" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>324</v>
       </c>
@@ -6607,9 +6616,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:AE19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>51</v>
       </c>
@@ -6632,7 +6641,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -6655,7 +6664,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
         <v>60</v>
       </c>
@@ -6664,19 +6673,19 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
         <v>61</v>
       </c>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>62</v>
       </c>
       <c r="D5" s="1"/>
     </row>
-    <row r="6" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="I6" s="1" t="s">
         <v>63</v>
       </c>
@@ -6688,7 +6697,7 @@
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
     </row>
-    <row r="7" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>64</v>
       </c>
@@ -6783,7 +6792,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="8" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>331</v>
       </c>
@@ -6854,7 +6863,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>339</v>
       </c>
@@ -6925,7 +6934,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>345</v>
       </c>
@@ -6996,7 +7005,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>352</v>
       </c>
@@ -7067,7 +7076,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>359</v>
       </c>
@@ -7138,7 +7147,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="13" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>366</v>
       </c>
@@ -7209,7 +7218,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>373</v>
       </c>
@@ -7280,7 +7289,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>379</v>
       </c>
@@ -7351,7 +7360,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>386</v>
       </c>
@@ -7422,7 +7431,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>393</v>
       </c>
@@ -7493,7 +7502,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>400</v>
       </c>
@@ -7564,7 +7573,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>406</v>
       </c>
@@ -7656,9 +7665,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:AE23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>51</v>
       </c>
@@ -7681,7 +7690,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -7704,7 +7713,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
         <v>60</v>
       </c>
@@ -7713,19 +7722,19 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
         <v>61</v>
       </c>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>62</v>
       </c>
       <c r="D5" s="1"/>
     </row>
-    <row r="6" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="I6" s="1" t="s">
         <v>63</v>
       </c>
@@ -7737,7 +7746,7 @@
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
     </row>
-    <row r="7" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>64</v>
       </c>
@@ -7832,7 +7841,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="8" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>414</v>
       </c>
@@ -7903,7 +7912,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>422</v>
       </c>
@@ -7974,7 +7983,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>428</v>
       </c>
@@ -8045,7 +8054,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>434</v>
       </c>
@@ -8116,7 +8125,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>440</v>
       </c>
@@ -8187,7 +8196,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="13" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>445</v>
       </c>
@@ -8258,7 +8267,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>454</v>
       </c>
@@ -8329,7 +8338,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>460</v>
       </c>
@@ -8400,7 +8409,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>467</v>
       </c>
@@ -8471,7 +8480,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>474</v>
       </c>
@@ -8542,7 +8551,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>481</v>
       </c>
@@ -8613,7 +8622,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>489</v>
       </c>
@@ -8684,7 +8693,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="20" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>496</v>
       </c>
@@ -8755,7 +8764,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="21" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>503</v>
       </c>
@@ -8826,7 +8835,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="22" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>508</v>
       </c>
@@ -8897,7 +8906,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="23" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>515</v>
       </c>
@@ -8989,9 +8998,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:AE15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>51</v>
       </c>
@@ -9014,7 +9023,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -9037,7 +9046,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
         <v>60</v>
       </c>
@@ -9046,19 +9055,19 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
         <v>61</v>
       </c>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>62</v>
       </c>
       <c r="D5" s="1"/>
     </row>
-    <row r="6" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="I6" s="1" t="s">
         <v>63</v>
       </c>
@@ -9070,7 +9079,7 @@
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
     </row>
-    <row r="7" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>64</v>
       </c>
@@ -9165,7 +9174,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="8" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>522</v>
       </c>
@@ -9236,7 +9245,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>530</v>
       </c>
@@ -9307,7 +9316,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>537</v>
       </c>
@@ -9378,7 +9387,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>543</v>
       </c>
@@ -9449,7 +9458,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>550</v>
       </c>
@@ -9520,7 +9529,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="13" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>557</v>
       </c>
@@ -9591,7 +9600,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>563</v>
       </c>
@@ -9662,7 +9671,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>570</v>
       </c>
@@ -9754,9 +9763,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:AE21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>51</v>
       </c>
@@ -9779,7 +9788,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -9802,7 +9811,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
         <v>60</v>
       </c>
@@ -9811,19 +9820,19 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
         <v>61</v>
       </c>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>62</v>
       </c>
       <c r="D5" s="1"/>
     </row>
-    <row r="6" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="I6" s="1" t="s">
         <v>63</v>
       </c>
@@ -9835,7 +9844,7 @@
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
     </row>
-    <row r="7" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>64</v>
       </c>
@@ -9930,7 +9939,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="8" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>577</v>
       </c>
@@ -10001,7 +10010,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>585</v>
       </c>
@@ -10072,7 +10081,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>591</v>
       </c>
@@ -10143,7 +10152,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>599</v>
       </c>
@@ -10214,7 +10223,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="12" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>610</v>
       </c>
@@ -10285,7 +10294,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="13" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>617</v>
       </c>
@@ -10356,7 +10365,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>624</v>
       </c>
@@ -10427,7 +10436,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>631</v>
       </c>
@@ -10498,7 +10507,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>638</v>
       </c>
@@ -10569,7 +10578,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>646</v>
       </c>
@@ -10640,7 +10649,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>654</v>
       </c>
@@ -10711,7 +10720,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>661</v>
       </c>
@@ -10782,7 +10791,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="20" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>669</v>
       </c>
@@ -10853,7 +10862,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="21" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>677</v>
       </c>
@@ -10945,9 +10954,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:R6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>685</v>
       </c>
@@ -11003,7 +11012,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>698</v>
       </c>
@@ -11059,7 +11068,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>254</v>
       </c>
@@ -11115,7 +11124,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>451</v>
       </c>
@@ -11171,7 +11180,7 @@
         <v>716</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>607</v>
       </c>
@@ -11227,7 +11236,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>615</v>
       </c>

</xml_diff>